<commit_message>
Conditional Formatting Applied on the table data
</commit_message>
<xml_diff>
--- a/Day 6/Employee_Data_Table.xlsx
+++ b/Day 6/Employee_Data_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5CB6121-5DF9-4719-9DA0-A98D781C03BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84BC266A-FBC7-44CA-BBCF-C6113211B1F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -239,7 +239,136 @@
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="14">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -837,6 +966,24 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F2:F11">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D11">
+    <cfRule type="top10" dxfId="5" priority="3" rank="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H11">
+    <cfRule type="timePeriod" dxfId="4" priority="2" timePeriod="nextWeek">
+      <formula>AND(ROUNDDOWN(H2,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(H2,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G11">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThanOrEqual">
+      <formula>100</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
More Conditional Formatting Applied on the table data using Color Scales and Icons Set
</commit_message>
<xml_diff>
--- a/Day 6/Employee_Data_Table.xlsx
+++ b/Day 6/Employee_Data_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84BC266A-FBC7-44CA-BBCF-C6113211B1F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{046187C2-F9CC-4DFD-9BEE-D4E8384FC0E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -239,7 +239,21 @@
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="22">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -268,9 +282,63 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -967,21 +1035,40 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F11">
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D11">
-    <cfRule type="top10" dxfId="5" priority="3" rank="5"/>
+    <cfRule type="top10" dxfId="6" priority="5" rank="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H11">
-    <cfRule type="timePeriod" dxfId="4" priority="2" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="5" priority="4" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(H2,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(H2,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G11">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThanOrEqual">
       <formula>100</formula>
+    </cfRule>
+    <cfRule type="iconSet" priority="1">
+      <iconSet iconSet="3Flags">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="33"/>
+        <cfvo type="percent" val="67"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E11">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>